<commit_message>
PivotTable Charts and Visuals
</commit_message>
<xml_diff>
--- a/Tewolde_Territory_Chart.xlsx
+++ b/Tewolde_Territory_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naomitewolde\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38A7C4ED-4B72-455C-AD21-2B838D6F2880}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{5FCFCE47-6E58-46FE-A383-81D270B5FC23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="3" xr2:uid="{F9E5F846-3F24-4A85-8C56-684E1499DFD8}"/>
   </bookViews>
@@ -206,9 +206,6 @@
     <t>Maryland Total Revenue</t>
   </si>
   <si>
-    <t xml:space="preserve">Notheast to Maryland Total Revenue </t>
-  </si>
-  <si>
     <t>Category Average Transaction Size</t>
   </si>
   <si>
@@ -228,6 +225,9 @@
   </si>
   <si>
     <t>State to Region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northeast to Maryland Total Revenue </t>
   </si>
 </sst>
 </file>
@@ -5218,7 +5218,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
@@ -5642,7 +5642,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -6381,10 +6381,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -6495,13 +6495,13 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="K1" s="20" t="s">
         <v>27</v>
-      </c>
-      <c r="E1" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="20" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
@@ -6618,10 +6618,10 @@
         <v>6</v>
       </c>
       <c r="R4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="S4" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.35">
@@ -6843,10 +6843,10 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10">
         <v>823</v>

</xml_diff>